<commit_message>
Update acceptance, validation, and get-well docs to current status
Reflect Li & Briggs two-stage road identification (Stage 1 complete,
Stage 2 in progress), auto-screenshot tool committed to GitHub, and
refreshed Sprint 2 target dates (completion target 11/02/2026).

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_017p6mccK4XQFabfMDvMtD8S
</commit_message>
<xml_diff>
--- a/docs/Sprint2-GetWell-Plan.xlsx
+++ b/docs/Sprint2-GetWell-Plan.xlsx
@@ -61,7 +61,7 @@
     <font>
       <name val="Arial"/>
       <b val="1"/>
-      <color rgb="00B45309"/>
+      <color rgb="00166534"/>
       <sz val="10"/>
     </font>
     <font>
@@ -182,7 +182,7 @@
     <xf numFmtId="0" fontId="5" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -557,7 +557,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F20"/>
+  <dimension ref="A1:F21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -727,7 +727,7 @@
       </c>
       <c r="D11" s="7" t="inlineStr">
         <is>
-          <t>Completed</t>
+          <t>Completed (on GitHub)</t>
         </is>
       </c>
     </row>
@@ -757,17 +757,17 @@
       </c>
       <c r="B13" s="9" t="inlineStr">
         <is>
-          <t>Requirements &amp; Design documents</t>
+          <t>Road identification Stage 1 — Li &amp; Briggs (linear-feature detection)</t>
         </is>
       </c>
       <c r="C13" s="8" t="inlineStr">
         <is>
-          <t>Vy</t>
+          <t>Don</t>
         </is>
       </c>
       <c r="D13" s="7" t="inlineStr">
         <is>
-          <t>Completed</t>
+          <t>Completed (on GitHub)</t>
         </is>
       </c>
     </row>
@@ -777,7 +777,7 @@
       </c>
       <c r="B14" s="6" t="inlineStr">
         <is>
-          <t>Definition of Done (Sprint 0 &amp; 1) + Acceptance / Validation docs</t>
+          <t>Requirements &amp; Design documents</t>
         </is>
       </c>
       <c r="C14" s="5" t="inlineStr">
@@ -797,128 +797,148 @@
       </c>
       <c r="B15" s="9" t="inlineStr">
         <is>
+          <t>Definition of Done (Sprint 0 &amp; 1) + Acceptance / Validation docs</t>
+        </is>
+      </c>
+      <c r="C15" s="8" t="inlineStr">
+        <is>
+          <t>Vy</t>
+        </is>
+      </c>
+      <c r="D15" s="7" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="26" customHeight="1">
+      <c r="A16" s="5" t="n">
+        <v>11</v>
+      </c>
+      <c r="B16" s="6" t="inlineStr">
+        <is>
           <t>Product Backlog + Trello board + Sprint 1 Retrospective</t>
         </is>
       </c>
-      <c r="C15" s="8" t="inlineStr">
+      <c r="C16" s="5" t="inlineStr">
         <is>
           <t>Vy</t>
         </is>
       </c>
-      <c r="D15" s="7" t="inlineStr">
+      <c r="D16" s="7" t="inlineStr">
         <is>
           <t>Completed</t>
         </is>
       </c>
     </row>
-    <row r="17" ht="22" customHeight="1">
-      <c r="A17" s="3" t="inlineStr">
+    <row r="18" ht="22" customHeight="1">
+      <c r="A18" s="3" t="inlineStr">
         <is>
           <t>2.  Planned Tasks NOT Completed — Carryover to Sprint 2</t>
         </is>
       </c>
     </row>
-    <row r="18">
-      <c r="A18" s="4" t="inlineStr">
+    <row r="19">
+      <c r="A19" s="4" t="inlineStr">
         <is>
           <t>Card</t>
         </is>
       </c>
-      <c r="B18" s="4" t="inlineStr">
+      <c r="B19" s="4" t="inlineStr">
         <is>
           <t>Task</t>
         </is>
       </c>
-      <c r="C18" s="4" t="inlineStr">
+      <c r="C19" s="4" t="inlineStr">
         <is>
           <t>Owner</t>
         </is>
       </c>
-      <c r="D18" s="4" t="inlineStr">
+      <c r="D19" s="4" t="inlineStr">
         <is>
           <t>Reason for Delay</t>
         </is>
       </c>
-      <c r="E18" s="4" t="inlineStr">
+      <c r="E19" s="4" t="inlineStr">
         <is>
           <t>Action Plan</t>
         </is>
       </c>
-      <c r="F18" s="4" t="inlineStr">
+      <c r="F19" s="4" t="inlineStr">
         <is>
           <t>Anticipated Completion</t>
         </is>
       </c>
     </row>
-    <row r="19" ht="96" customHeight="1">
-      <c r="A19" s="10" t="inlineStr">
+    <row r="20" ht="96" customHeight="1">
+      <c r="A20" s="10" t="inlineStr">
         <is>
           <t>S1-8-B</t>
         </is>
       </c>
-      <c r="B19" s="6" t="inlineStr">
+      <c r="B20" s="6" t="inlineStr">
         <is>
           <t>Road Mapping Coordinate-finding System</t>
         </is>
       </c>
-      <c r="C19" s="5" t="inlineStr">
+      <c r="C20" s="5" t="inlineStr">
         <is>
           <t>Don (DF)</t>
         </is>
       </c>
-      <c r="D19" s="11" t="inlineStr">
-        <is>
-          <t>The initial scikit-image approach (contrast + morphology + pixel trace) could not reliably isolate road geometry — shadow/tree noise and broken road continuity. Testing also showed NJGIN overhead resolution limits fine detail.</t>
-        </is>
-      </c>
-      <c r="E19" s="12" t="inlineStr">
-        <is>
-          <t>Move to Sprint 2. Pivot to a published road-extraction method (Li &amp; Briggs, 2009); re-implement isolation and output road/segment coordinates. Rough-coordinate algorithm is retained.</t>
-        </is>
-      </c>
-      <c r="F19" s="5" t="inlineStr">
-        <is>
-          <t>Sprint 2 — Wk 2 (target 10/29/2026)</t>
-        </is>
-      </c>
-    </row>
-    <row r="20" ht="96" customHeight="1">
-      <c r="A20" s="13" t="inlineStr">
+      <c r="D20" s="11" t="inlineStr">
+        <is>
+          <t>In progress. Road identification was re-approached with the published Li &amp; Briggs two-stage method. Stage 1 (linear-feature detection / grouping) is complete and committed to GitHub; Stage 2 (asphalt spectral-signature resweep + tree/railroad rejection) and local-pixel→lat/long georeferencing remain before coordinates can be written to the DB.</t>
+        </is>
+      </c>
+      <c r="E20" s="12" t="inlineStr">
+        <is>
+          <t>Move to Sprint 2. Finish Stage 2, georeference using the sector corner lat/longs (local → global), and output road/segment coordinates to the DB. Rough-coordinate algorithm is retained.</t>
+        </is>
+      </c>
+      <c r="F20" s="5" t="inlineStr">
+        <is>
+          <t>Sprint 2 — Wk 1 (target 10/26/2026)</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="96" customHeight="1">
+      <c r="A21" s="13" t="inlineStr">
         <is>
           <t>S1-8</t>
         </is>
       </c>
-      <c r="B20" s="9" t="inlineStr">
+      <c r="B21" s="9" t="inlineStr">
         <is>
           <t>Database Population B; Road/Segment-level Population &amp; Auto-Screenshot</t>
         </is>
       </c>
-      <c r="C20" s="8" t="inlineStr">
+      <c r="C21" s="8" t="inlineStr">
         <is>
           <t>Vy, Cristofer, Don (VK/CS/DF)</t>
         </is>
       </c>
-      <c r="D20" s="11" t="inlineStr">
-        <is>
-          <t>Blocked on S1-8-B: the auto-screenshot tool is complete, but road/segment-level capture needs the coordinates from the coordinate-finding system to know where to capture. Could not start population without them.</t>
-        </is>
-      </c>
-      <c r="E20" s="14" t="inlineStr">
+      <c r="D21" s="11" t="inlineStr">
+        <is>
+          <t>Blocked on S1-8-B coordinate output. The auto-screenshot tool is complete and committed to GitHub; road/segment-level capture needs the coordinates from Stage 2 to know where to capture, so population could not start.</t>
+        </is>
+      </c>
+      <c r="E21" s="14" t="inlineStr">
         <is>
           <t>Move to Sprint 2 (after S1-8-B). Batch-run auto-screenshot across sector/road/segment coordinates, then load image file locations into the DB and verify.</t>
         </is>
       </c>
-      <c r="F20" s="8" t="inlineStr">
-        <is>
-          <t>Sprint 2 — end (target 11/05/2026)</t>
+      <c r="F21" s="8" t="inlineStr">
+        <is>
+          <t>Sprint 2 (target 11/02/2026)</t>
         </is>
       </c>
     </row>
   </sheetData>
   <mergeCells count="4">
     <mergeCell ref="A2:F2"/>
-    <mergeCell ref="A17:F17"/>
     <mergeCell ref="A1:F1"/>
+    <mergeCell ref="A18:F18"/>
     <mergeCell ref="A4:F4"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -955,10 +975,10 @@
         </is>
       </c>
     </row>
-    <row r="4" ht="28" customHeight="1">
+    <row r="4" ht="44" customHeight="1">
       <c r="A4" s="15" t="inlineStr">
         <is>
-          <t>Dependency: S1-8-B (coordinates) must finish before S1-8 (population) can run.  They are sequenced, not parallel.</t>
+          <t>Current progress (10/16):  Road identification Stage 1 (Li &amp; Briggs linear-feature detection) is complete and committed; Stage 2 is in progress.  The auto-screenshot tool is complete and on GitHub.  Dependency: S1-8-B (coordinates) must finish before S1-8 (population) can run — sequenced, not parallel.</t>
         </is>
       </c>
     </row>
@@ -1011,7 +1031,7 @@
       </c>
       <c r="B9" s="12" t="inlineStr">
         <is>
-          <t>Implement the Li &amp; Briggs (2009) road-extraction method on sample NJGIN sectors (replace the scikit-image isolation step).</t>
+          <t>Finish Stage 2 — learn the asphalt spectral signature under the Stage-1 segments, resweep to recover missing roads, and add checks to reject trees / railroad tracks.</t>
         </is>
       </c>
       <c r="C9" s="5" t="inlineStr">
@@ -1021,12 +1041,12 @@
       </c>
       <c r="D9" s="12" t="inlineStr">
         <is>
-          <t>Method runs on a sector tile and outputs a clean road mask.</t>
+          <t>Stage 2 recovers missing roads and rejects non-road linear features on a sample sector.</t>
         </is>
       </c>
       <c r="E9" s="5" t="inlineStr">
         <is>
-          <t>10/22/2026</t>
+          <t>10/20/2026</t>
         </is>
       </c>
     </row>
@@ -1038,7 +1058,7 @@
       </c>
       <c r="B10" s="14" t="inlineStr">
         <is>
-          <t>Validate centerline / coordinate output on 3–5 known roads; tune thresholds.</t>
+          <t>Georeference — use the sector corner lat/longs to translate local (in-sector) pixel coordinates to global lat/long.</t>
         </is>
       </c>
       <c r="C10" s="8" t="inlineStr">
@@ -1048,12 +1068,12 @@
       </c>
       <c r="D10" s="14" t="inlineStr">
         <is>
-          <t>Extracted road lines match the real roads on known samples.</t>
+          <t>A road's pixels map to the correct real-world lat/long on a known sector.</t>
         </is>
       </c>
       <c r="E10" s="8" t="inlineStr">
         <is>
-          <t>10/26/2026</t>
+          <t>10/23/2026</t>
         </is>
       </c>
     </row>
@@ -1080,7 +1100,7 @@
       </c>
       <c r="E11" s="5" t="inlineStr">
         <is>
-          <t>10/29/2026</t>
+          <t>10/26/2026</t>
         </is>
       </c>
     </row>
@@ -1148,7 +1168,7 @@
       </c>
       <c r="E16" s="5" t="inlineStr">
         <is>
-          <t>11/01/2026</t>
+          <t>10/28/2026</t>
         </is>
       </c>
     </row>
@@ -1175,7 +1195,7 @@
       </c>
       <c r="E17" s="8" t="inlineStr">
         <is>
-          <t>11/03/2026</t>
+          <t>10/30/2026</t>
         </is>
       </c>
     </row>
@@ -1202,14 +1222,14 @@
       </c>
       <c r="E18" s="5" t="inlineStr">
         <is>
-          <t>11/05/2026</t>
+          <t>11/02/2026</t>
         </is>
       </c>
     </row>
     <row r="20" ht="24" customHeight="1">
       <c r="A20" s="18" t="inlineStr">
         <is>
-          <t>Anticipated full completion of both carryover tasks:  end of Sprint 2 — target 11/05/2026.</t>
+          <t>Anticipated full completion of both carryover tasks:  target 11/02/2026 (Sprint 2).</t>
         </is>
       </c>
     </row>

</xml_diff>